<commit_message>
Publish review control set and workbooks through CLS-05
</commit_message>
<xml_diff>
--- a/review/abilities/workbooks/00_Index_and_Review_Findings.xlsx
+++ b/review/abilities/workbooks/00_Index_and_Review_Findings.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Inventory" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Findings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Flagged Cards" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Change Log" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Coverage" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Method" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flagged Cards" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inventory'!$A$4:$E$23</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Inventory'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$4:$I$36</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Findings'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Flagged Cards'!$A$4:$J$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Flagged Cards'!$A$4:$J$99</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Flagged Cards'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Change Log'!$A$4:$R$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Change Log'!$A$4:$Q$204</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Change Log'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Change Log'!$A$1:$R$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Change Log'!$A$1:$Q$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -284,7 +284,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="4">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -321,19 +321,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00F8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-        <b val="1"/>
-        <color rgb="001F3864"/>
-        <sz val="9"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00D9E1F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -713,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -830,7 +817,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>32 (6 High, 13 Medium, 11 Low, 2 Positive)</t>
+          <t>32 (6 High, 12 Medium, 11 Low, 3 Positive)</t>
         </is>
       </c>
     </row>
@@ -842,7 +829,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>96 cards with at least one row-level flag</t>
+          <t>95 cards with at least one row-level flag</t>
         </is>
       </c>
     </row>
@@ -877,7 +864,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>• Use the Decision column (Keep / Revise / Cut / Playtest / Unsure) and Your notes. The dropdown is already installed on every data sheet.</t>
+          <t>• Use the Decision column (Keep / Revise / Cut / Unsure) and Your notes. The dropdown is already installed on every data sheet.</t>
         </is>
       </c>
     </row>
@@ -953,85 +940,74 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Playtest</t>
+          <t>Unsure</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>The idea is sound but needs table evidence before a change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Unsure</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
           <t>Needs more information or a design decision outside this review.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Start here: the highest-value decisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>• F02 — Eight shared cards have no discipline requirement beyond the six stated 1-DP exceptions: seven 2-DP Novice skill cards and One More Dawn (Master, 8 DP).</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>• F02 — Eight shared cards have no discipline requirement beyond the six stated 1-DP exceptions: seven 2-DP Novice skill cards and One More Dawn (Master, 8 DP).</t>
+          <t>• F03 — Master tier, 8 DP, no requirement, once-ever +1 Grit that never replenishes spent Grit.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>• F03 — Master tier, 8 DP, no requirement, once-ever +1 Grit that never replenishes spent Grit.</t>
+          <t>• F04 — Repeatable +1 maximum HP, one purchase allowed at each level, no upper cap and no discipline requirement.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>• F04 — Repeatable +1 maximum HP, one purchase allowed at each level, no upper cap and no discipline requirement.</t>
+          <t>• F05 — Master tier, 8 DP, Armor 3, Reaction solely to 'remain standing' when an effect would knock you prone.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>• F05 — Master tier, 8 DP, Armor 3, Reaction solely to 'remain standing' when an effect would knock you prone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
+          <t>• F06 — Requires 'Craft 1; known compatible crafting card', a card prerequisite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="32" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>• F06 — Requires 'Craft 1; known compatible crafting card', a card prerequisite.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="32" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
           <t>• F07 — Near-duplicate cards: both are Craft 1, 2 DP, Main Action, Knowledge, grant tools and two ordinary recipes, use the same recipe list and produce the same 1/2/3 progress outcomes. The substantive difference is salvage substitution and a Strong rider on Make Something Useful.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="9" t="inlineStr">
-        <is>
-          <t>Generated 2026-10-23 from the read-only reference repository. Source markdown was not modified.</t>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>Generated 2026-10-26 from the read-only reference repository. Source markdown was not modified.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="33">
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="B31:F31"/>
@@ -1039,8 +1015,8 @@
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
     <mergeCell ref="B12:F12"/>
-    <mergeCell ref="A42:F42"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="A23:F23"/>
@@ -1056,7 +1032,6 @@
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A40:F40"/>
     <mergeCell ref="A39:F39"/>
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="B30:F30"/>
@@ -1064,7 +1039,6 @@
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="B32:F32"/>
     <mergeCell ref="A7:F7"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -1153,7 +1127,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>32 findings / 96 flags</t>
+          <t>32 findings / 95 flags</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -2209,17 +2183,17 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Halfling is HP +1 and Speed 5 with no trait that raises HP or Speed. Dwarf can reach HP +5, Human HP +3 or Speed 7, Elf Speed 7. Halfling's traits are mostly situational except A Little Luck.</t>
+          <t>Halfling is HP +1 and Speed 5. Bigger on the Inside now raises HP, but no Halfling trait raises Speed, and the ancestry still has the lowest base HP/Speed.</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Halfling is the weakest ancestry on raw statistics, and its best trait is a once-per-day generic Boon. That may be intentional, but it is not explained.</t>
+          <t>The HP trait closes part of the raw-stat gap, but Halfling remains the slowest ancestry and has no Speed trait. A Little Luck is still its broadest trait.</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>Add +1 maximum HP to Bigger on the Inside or Second Breakfast, or give Under Their Noses a broader always-on benefit. If the gap is intentional, state the compensation (luck/stealth) in the ancestry text.</t>
+          <t>Keep the +1 HP on Bigger on the Inside. Consider a Speed trait or a small always-on movement benefit if Halfling still feels slow. If the gap is intentional, state the luck/stealth compensation in the ancestry text.</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
@@ -2229,10 +2203,10 @@
       </c>
       <c r="I15" s="10" t="inlineStr"/>
     </row>
-    <row r="16" ht="66.5" customHeight="1">
+    <row r="16" ht="54" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>F12</t>
+          <t>F13</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -2242,27 +2216,27 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Ancestry</t>
+          <t>Ancestry / Halfling</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Stubborn as Bedrock; Never Quite Finished; Grace of the Elder Folk; Road in the Blood</t>
+          <t>A Little Luck</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Two pairs of ancestry traits are mechanically identical: Stubborn as Bedrock and Never Quite Finished are both '+1 maximum HP'; Grace of the Elder Folk and Road in the Blood are both '+1 base Speed'.</t>
+          <t>Once per day, before any attribute roll, gain 1 Boon. This is the broadest ancestry trait in the game.</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Reduces ancestry distinctiveness and makes two trait choices feel like the same pick with different flavor.</t>
+          <t>Likely the Halfling default pick. It can apply to attacks, defenses and any skill, unlike most traits which are narrow.</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Keep the stat but add a small ancestry-specific rider: Dwarf +1 to stabilization or reduce Bleeding after a rest; Human a travel/endurance clause; Elf ignore 1 square of difficult terrain once per scene; Human speed a forced-march benefit.</t>
+          <t>Monitor at the table. If it dominates, make it once per scene, require a roll with a meaningful consequence, or limit it to non-attack rolls. Keep it if Halfling needs the power (see F11).</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -2275,7 +2249,7 @@
     <row r="17" ht="54" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>F13</t>
+          <t>F14</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
@@ -2285,27 +2259,27 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Ancestry / Halfling</t>
+          <t>Universal</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>A Little Luck</t>
+          <t>Command a Summon; Convert an Action; Handle an Item</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Once per day, before any attribute roll, gain 1 Boon. This is the broadest ancestry trait in the game.</t>
+          <t>Three universal cards use action labels outside the five standard labels: 'Main Action or Maneuver', 'Action conversion' and 'Varies'.</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Likely the Halfling default pick. It can apply to attacks, defenses and any skill, unlike most traits which are narrow.</t>
+          <t>The conventions state that Main Action, Maneuver, Reaction, Movement and Passive are distinct labels. These three break VTT sorting, print layout and quick reference.</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>Monitor at the table. If it dominates, make it once per scene, require a roll with a meaningful consequence, or limit it to non-attack rolls. Keep it if Halfling needs the power (see F11).</t>
+          <t>Add a secondary 'Action detail' field for compound costs, or define the labels in the conventions. Convert an Action reads like a rules procedure, not an ability; consider moving it to the combat chapter.</t>
         </is>
       </c>
       <c r="H17" s="10" t="inlineStr">
@@ -2318,7 +2292,7 @@
     <row r="18" ht="54" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>F14</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -2333,22 +2307,22 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Command a Summon; Convert an Action; Handle an Item</t>
+          <t>Basic Melee; Basic Ranged; Basic Throw; Basic Unarmed</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Three universal cards use action labels outside the five standard labels: 'Main Action or Maneuver', 'Action conversion' and 'Varies'.</t>
+          <t>The four basic attacks have Tier Universal but Type Attack; the other fourteen universal cards have Type Universal.</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>The conventions state that Main Action, Maneuver, Reaction, Movement and Passive are distinct labels. These three break VTT sorting, print layout and quick reference.</t>
+          <t>A Type = Universal filter returns 14, not 18. 'Universal' is doing double duty as a tier and a type, so counts and indexes will disagree.</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Add a secondary 'Action detail' field for compound costs, or define the labels in the conventions. Convert an Action reads like a rules procedure, not an ability; consider moving it to the combat chapter.</t>
+          <t>Make Type functional (Attack, Defense, Movement, Utility) for all cards and let Tier/availability carry 'Universal'; or add a Universal tag to the four attacks and document the distinction.</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -2358,10 +2332,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
     </row>
-    <row r="19" ht="54" customHeight="1">
+    <row r="19" ht="79" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>F16</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
@@ -2371,27 +2345,27 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Universal</t>
+          <t>Master</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Basic Melee; Basic Ranged; Basic Throw; Basic Unarmed</t>
+          <t>A Company of Reflections; A Voice across the Valley; Four Winds at Once</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>The four basic attacks have Tier Universal but Type Attack; the other fourteen universal cards have Type Universal.</t>
+          <t>Three Master cards require only two rank-2 disciplines (Mind 2 + Guard 2; Mind 2 + Storm 2; Storm 2 + Athletics 2).</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>A Type = Universal filter returns 14, not 18. 'Universal' is doing double duty as a tier and a type, so counts and indexes will disagree.</t>
+          <t>Two rank-2 disciplines cost 6 discipline DP before class pricing; one rank-3 discipline costs 7. These Master effects are therefore cheaper to access than a specialist Master card. That may be the intended cross-training route, but it is not stated.</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>Make Type functional (Attack, Defense, Movement, Utility) for all cards and let Tier/availability carry 'Universal'; or add a Universal tag to the four attacks and document the distinction.</t>
+          <t>Confirm the intent. If these are meant to be broad Master options, add a policy note. If not, raise one requirement to rank 3. A Voice across the Valley is also noncombat utility; consider Adept if it is not meant to be a Master capstone.</t>
         </is>
       </c>
       <c r="H19" s="10" t="inlineStr">
@@ -2401,10 +2375,10 @@
       </c>
       <c r="I19" s="10" t="inlineStr"/>
     </row>
-    <row r="20" ht="79" customHeight="1">
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>F16</t>
+          <t>F17</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
@@ -2414,27 +2388,27 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Master</t>
+          <t>All tiers</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>A Company of Reflections; A Voice across the Valley; Four Winds at Once</t>
+          <t>Close Shot; Find the Seam; Sell the Feint; Take the Measure; Wind the Sight</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Three Master cards require only two rank-2 disciplines (Mind 2 + Guard 2; Mind 2 + Storm 2; Storm 2 + Athletics 2).</t>
+          <t>Five shared cards carry Type Skill / Attack but make no attack roll; they only set up or improve a later attack.</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>Two rank-2 disciplines cost 6 discipline DP before class pricing; one rank-3 discipline costs 7. These Master effects are therefore cheaper to access than a specialist Master card. That may be the intended cross-training route, but it is not stated.</t>
+          <t>Attack filters and quick-reference tables imply an attack that the card does not make. The same ambiguity appears in signature tags, where attack riders often lack the Attack tag.</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Confirm the intent. If these are meant to be broad Master options, add a policy note. If not, raise one requirement to rank 3. A Voice across the Valley is also noncombat utility; consider Adept if it is not meant to be a Master capstone.</t>
+          <t>Add a Setup tag for attack-support cards, or document that Attack includes 'sets up an attack'. Apply the same rule to signature Tags so the taxonomy is predictable.</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2444,10 +2418,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
     </row>
-    <row r="21" ht="54" customHeight="1">
+    <row r="21" ht="66.5" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>F17</t>
+          <t>F18</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
@@ -2457,40 +2431,40 @@
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>All tiers</t>
+          <t>Class signatures</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Close Shot; Find the Seam; Sell the Feint; Take the Measure; Wind the Sight</t>
+          <t>Between Them; Follow My Signal; Return Stroke; Relentless Pursuit; Unseen Passage; Unbroken Passage; A Watchful Rest; A Route for Everyone; Arcane Deflection; Watch the Rear</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Five shared cards carry Type Skill / Attack but make no attack roll; they only set up or improve a later attack.</t>
+          <t>Ten signature abilities are clear power spikes: a level-1 intercept, Aid for two allies, repeatable free attacks, a round of untargetability, party-wide movement, an 8-hour watch buff, and 2-Boon reactions.</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>Attack filters and quick-reference tables imply an attack that the card does not make. The same ambiguity appears in signature tags, where attack riders often lack the Attack tag.</t>
+          <t>These are likely auto-picks and can dominate spotlight/action economy. They may be intentional class fantasies, but they need playtest attention and clear limits.</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>Add a Setup tag for attack-support cards, or document that Attack includes 'sets up an attack'. Apply the same rule to signature Tags so the taxonomy is predictable.</t>
+          <t>Playtest these first. Consider once-per-round limits, adjacency requirements, shorter durations, or 1 Boon instead of 2 where the spike is largest. Keep the fantasy; tighten the repeatability.</t>
         </is>
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="I21" s="10" t="inlineStr"/>
     </row>
-    <row r="22" ht="66.5" customHeight="1">
+    <row r="22" ht="54" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>F18</t>
+          <t>F19</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
@@ -2505,22 +2479,22 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Between Them; Follow My Signal; Return Stroke; Relentless Pursuit; Unseen Passage; Unbroken Passage; A Watchful Rest; A Route for Everyone; Arcane Deflection; Watch the Rear</t>
+          <t>Choose the Edge; Perfect Placement; Break Their Grip; Open the Way; Leave No Pursuit</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Ten signature abilities are clear power spikes: a level-1 intercept, Aid for two allies, repeatable free attacks, a round of untargetability, party-wide movement, an 8-hour watch buff, and 2-Boon reactions.</t>
+          <t>Several Master or Adept signature choices are simple riders or narrow utility: a 2-square push, a 2-square push plus move, an anti-grapple maneuver, a lockpicking card and a trail-concealment card.</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>These are likely auto-picks and can dominate spotlight/action economy. They may be intentional class fantasies, but they need playtest attention and clear limits.</t>
+          <t>A signature slot is precious. Narrow or incremental options may never be chosen over broader class-defining abilities.</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Playtest these first. Consider once-per-round limits, adjacency requirements, shorter durations, or 1 Boon instead of 2 where the spike is largest. Keep the fantasy; tighten the repeatability.</t>
+          <t>For each, either add a second clause that broadens the moment (condition, ally benefit, alternate use) or accept it as a deliberate specialist pick and say so in the class guidance.</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2533,42 +2507,42 @@
     <row r="23" ht="54" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>F19</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>F20</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Class signatures</t>
+          <t>Universal</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Choose the Edge; Perfect Placement; Break Their Grip; Open the Way; Leave No Pursuit</t>
+          <t>Force; Strange but Effective</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Several Master or Adept signature choices are simple riders or narrow utility: a 2-square push, a 2-square push plus move, an anti-grapple maneuver, a lockpicking card and a trail-concealment card.</t>
+          <t>Outcome lines read '2 progress, grapple reduction, or squares of push' and '3 progress, Grappled reduction, or squares of push'; the push numeral is missing in five lines across the two cards.</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>A signature slot is precious. Narrow or incremental options may never be chosen over broader class-defining abilities.</t>
+          <t>Ambiguous push distance. The intended values are inferable (Force 1/2/3; Strange 2/3/4) but not printed.</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>For each, either add a second clause that broadens the moment (condition, ally benefit, alternate use) or accept it as a deliberate specialist pick and say so in the class guidance.</t>
+          <t>Write the numeral every time: 'or 1 square of push', 'or 2 squares of push', etc. Check other multi-option outcome lines for the same pattern.</t>
         </is>
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr"/>
@@ -2576,7 +2550,7 @@
     <row r="24" ht="54" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>F20</t>
+          <t>F21</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2591,22 +2565,22 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Force; Strange but Effective</t>
+          <t>Stabilize; Command a Summon; Opportunity Attack; Aid</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Outcome lines read '2 progress, grapple reduction, or squares of push' and '3 progress, Grappled reduction, or squares of push'; the push numeral is missing in five lines across the two cards.</t>
+          <t>Four wording issues: 'Stabilize at 0 HP' lacks an object; 'within its tether' is ambiguous; Opportunity Attack's Attribute field contains a sentence; Aid still says 'Proposal:'.</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Ambiguous push distance. The intended values are inferable (Force 1/2/3; Strange 2/3/4) but not printed.</t>
+          <t>Small clarity issues in the most-used universal actions, where every table will read them.</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Write the numeral every time: 'or 1 square of push', 'or 2 squares of push', etc. Check other multi-option outcome lines for the same pattern.</t>
+          <t>Rewrite: 'Stabilize a Dying character at 0 HP'; 'within 6 squares of you (its tether)'; Attribute 'Brawn (no separate roll)'; remove 'Proposal:'.</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2619,7 +2593,7 @@
     <row r="25" ht="54" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>F21</t>
+          <t>F22</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2629,27 +2603,27 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Universal</t>
+          <t>All tiers</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Stabilize; Command a Summon; Opportunity Attack; Aid</t>
+          <t>Multiple</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Four wording issues: 'Stabilize at 0 HP' lacks an object; 'within its tether' is ambiguous; Opportunity Attack's Attribute field contains a sentence; Aid still says 'Proposal:'.</t>
+          <t>Type and Tag ordering is inconsistent: 'Magic / Utility / Control' vs 'Magic / Control / Utility'; 'Skill / Movement / Defense' vs 'Skill / Defense / Movement'; signature Tags have the same issue.</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>Small clarity issues in the most-used universal actions, where every table will read them.</t>
+          <t>Filters, grouping and VTT tag sets treat equivalent cards as different strings.</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>Rewrite: 'Stabilize a Dying character at 0 HP'; 'within 6 squares of you (its tether)'; Attribute 'Brawn (no separate roll)'; remove 'Proposal:'.</t>
+          <t>Normalize to a canonical order (alphabetical or the order in card-conventions) at build time and in the source files.</t>
         </is>
       </c>
       <c r="H25" s="10" t="inlineStr">
@@ -2662,7 +2636,7 @@
     <row r="26" ht="54" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>F22</t>
+          <t>F23</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2672,27 +2646,27 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>All tiers</t>
+          <t>Ancestry</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Multiple</t>
+          <t>All 20 ancestry traits</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Type and Tag ordering is inconsistent: 'Magic / Utility / Control' vs 'Magic / Control / Utility'; 'Skill / Movement / Defense' vs 'Skill / Defense / Movement'; signature Tags have the same issue.</t>
+          <t>Trait filenames/IDs no longer match current titles: trait-dwarf-deep-constitution is 'Hard as Bedrock'; trait-human-weathered is 'The Impossible Streak'; trait-halfling-good-cheer is 'Make Room at the Fire'.</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>Filters, grouping and VTT tag sets treat equivalent cards as different strings.</t>
+          <t>Stable IDs are good for links, but editors and reviewers cannot find a trait by filename. The mismatch is invisible in the catalog.</t>
         </is>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Normalize to a canonical order (alphabetical or the order in card-conventions) at build time and in the source files.</t>
+          <t>Keep stable IDs, but add a 'Source file' column in review workbooks and document the naming policy. If IDs can change before release, align them now.</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2702,10 +2676,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
     </row>
-    <row r="27" ht="54" customHeight="1">
+    <row r="27" ht="41.5" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>F23</t>
+          <t>F24</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2715,27 +2689,27 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Ancestry</t>
+          <t>Class / Warden</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>All 20 ancestry traits</t>
+          <t>Warden class file</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>Trait filenames/IDs no longer match current titles: trait-dwarf-deep-constitution is 'Stubborn as Bedrock'; trait-human-weathered is 'The Impossible Streak'; trait-halfling-good-cheer is 'Make Room at the Fire'.</t>
+          <t>Warden uses 'Class foundations' instead of 'Agreed' and has no 'Signature identity in play' section, unlike the other nine classes.</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>Stable IDs are good for links, but editors and reviewers cannot find a trait by filename. The mismatch is invisible in the catalog.</t>
+          <t>The class reads as a different template and the signature guidance is missing from the player-facing page.</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>Keep stable IDs, but add a 'Source file' column in review workbooks and document the naming policy. If IDs can change before release, align them now.</t>
+          <t>Standardize the heading and add the same signature-identity bullets used by the other classes.</t>
         </is>
       </c>
       <c r="H27" s="10" t="inlineStr">
@@ -2745,10 +2719,10 @@
       </c>
       <c r="I27" s="10" t="inlineStr"/>
     </row>
-    <row r="28" ht="41.5" customHeight="1">
+    <row r="28" ht="79" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>F24</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2758,27 +2732,27 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Class / Warden</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Warden class file</t>
+          <t>A Bough for the Fallen; Mercy in the Light; Return to Strength; Sap and Breath; Shared Breath; Stitch the Living Pattern; Sustain the Failing; Careful Transfer; Restore Composure; Catch a Falling Friend; Haul Them Home</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Warden uses 'Class foundations' instead of 'Agreed' and has no 'Signature identity in play' section, unlike the other nine classes.</t>
+          <t>Nine cards carry an 'Offensive healing — latest agreement' footnote and two carry a 'Stability exception' footnote, all placed after the card links rather than inside Rules.</t>
         </is>
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>The class reads as a different template and the signature guidance is missing from the player-facing page.</t>
+          <t>These are important exceptions that change targeting and movement. Players reading only the Rules block can miss them.</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Standardize the heading and add the same signature-identity bullets used by the other classes.</t>
+          <t>Move each exception into the Rules section as a short paragraph, or add a keyword/tag ('Harmful healing', 'Stability exception') and index it.</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2788,10 +2762,10 @@
       </c>
       <c r="I28" s="11" t="inlineStr"/>
     </row>
-    <row r="29" ht="79" customHeight="1">
+    <row r="29" ht="41.5" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F26</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2801,27 +2775,27 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Recovery</t>
+          <t>Classes</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>A Bough for the Fallen; Mercy in the Light; Return to Strength; Sap and Breath; Shared Breath; Stitch the Living Pattern; Sustain the Failing; Careful Transfer; Restore Composure; Catch a Falling Friend; Haul Them Home</t>
+          <t>All 10 classes</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>Nine cards carry an 'Offensive healing — latest agreement' footnote and two carry a 'Stability exception' footnote, all placed after the card links rather than inside Rules.</t>
+          <t>Starting coin contributions range from +0 (Odd, Unbalanced) to +8 (Intellect), while total starting purses stay within the documented 50-70 coin band.</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>These are important exceptions that change targeting and movement. Players reading only the Rules block can miss them.</t>
+          <t>The spread is deliberate and documented, but it can look unequal at session one without the starting-coins explanation.</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>Move each exception into the Rules section as a short paragraph, or add a keyword/tag ('Harmful healing', 'Stability exception') and index it.</t>
+          <t>No mechanical change. Mention the purse range and the reason for class contributions in each class overview, and point to starting-coins.md.</t>
         </is>
       </c>
       <c r="H29" s="10" t="inlineStr">
@@ -2831,10 +2805,10 @@
       </c>
       <c r="I29" s="10" t="inlineStr"/>
     </row>
-    <row r="30" ht="41.5" customHeight="1">
+    <row r="30" ht="54" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>F26</t>
+          <t>F27</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -2844,27 +2818,27 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Classes</t>
+          <t>Universal</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>All 10 classes</t>
+          <t>Basic Melee; Basic Ranged; Basic Throw; Basic Unarmed</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Starting coin contributions range from +0 (Odd, Unbalanced) to +8 (Intellect), while total starting purses stay within the documented 50-70 coin band.</t>
+          <t>The basic attack hierarchy is Unarmed 1/2/4, Throw and Ranged 2/3/5, Melee 2/4/6.</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>The spread is deliberate and documented, but it can look unequal at session one without the starting-coins explanation.</t>
+          <t>Melee is strictly the highest damage baseline; thrown and ranged are equal; unarmed is lowest. That may be intended, but it is not stated in one place.</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>No mechanical change. Mention the purse range and the reason for class contributions in each class overview, and point to starting-coins.md.</t>
+          <t>Add a short designer's note in the universal overview and in the combat chapter so players understand the baseline before choosing attack cards.</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2877,7 +2851,7 @@
     <row r="31" ht="54" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>F27</t>
+          <t>F30</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -2887,113 +2861,113 @@
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
+          <t>Ancestry</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>All ancestries</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>All 20 ancestry traits are Passive; none asks for an action or a roll of its own.</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Ancestry choice is a set of always-on modifiers, which keeps character creation simple but means ancestry never provides an active option in play.</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>This is a coherent design choice; keep it. If more ancestry texture is wanted, add one active once-per-scene trait per ancestry rather than converting existing passives.</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32" ht="66.5" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Class signatures</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Make the Connection; Test the Hypothesis; Expose the Mechanism; Know What You Hunt</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Two signature pairs occupy similar niches: Intellect's Make the Connection and Test the Hypothesis are both evidence analysis, and Intellect's Expose the Mechanism and Warden's Know What You Hunt both reveal a target's resistances/weaknesses and grant allies Boons.</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>Class identity can blur, and a DA may let one class's signature substitute for another's. The Master versions need to feel clearly larger than the lower-tier versions.</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>Differentiate by time and scope: Intellect reads the immediate scene; Warden knows the quarry over a hunt. Make the Master investigation (Test the Hypothesis) clearly bigger than the one-minute version. State the intended overlap in the class guidance if it is deliberate.</t>
+        </is>
+      </c>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr"/>
+    </row>
+    <row r="33" ht="54" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
           <t>Universal</t>
         </is>
       </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>Basic Melee; Basic Ranged; Basic Throw; Basic Unarmed</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>The basic attack hierarchy is Unarmed 1/2/4, Throw and Ranged 2/3/5, Melee 2/4/6.</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Melee is strictly the highest damage baseline; thrown and ranged are equal; unarmed is lowest. That may be intended, but it is not stated in one place.</t>
-        </is>
-      </c>
-      <c r="G31" s="10" t="inlineStr">
-        <is>
-          <t>Add a short designer's note in the universal overview and in the combat chapter so players understand the baseline before choosing attack cards.</t>
-        </is>
-      </c>
-      <c r="H31" s="10" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I31" s="10" t="inlineStr"/>
-    </row>
-    <row r="32" ht="54" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>F30</t>
-        </is>
-      </c>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>Ancestry</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>All ancestries</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="inlineStr">
-        <is>
-          <t>All 20 ancestry traits are Passive; none asks for an action or a roll of its own.</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>Ancestry choice is a set of always-on modifiers, which keeps character creation simple but means ancestry never provides an active option in play.</t>
-        </is>
-      </c>
-      <c r="G32" s="11" t="inlineStr">
-        <is>
-          <t>This is a coherent design choice; keep it. If more ancestry texture is wanted, add one active once-per-scene trait per ancestry rather than converting existing passives.</t>
-        </is>
-      </c>
-      <c r="H32" s="11" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr"/>
-    </row>
-    <row r="33" ht="66.5" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>F31</t>
-        </is>
-      </c>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>Class signatures</t>
-        </is>
-      </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>Make the Connection; Test the Hypothesis; Expose the Mechanism; Know What You Hunt</t>
+          <t>All 18 universal cards</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>Two signature pairs occupy similar niches: Intellect's Make the Connection and Test the Hypothesis are both evidence analysis, and Intellect's Expose the Mechanism and Warden's Know What You Hunt both reveal a target's resistances/weaknesses and grant allies Boons.</t>
+          <t>Universal cards store DP as the text 'Not purchased' instead of 0 or blank.</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>Class identity can blur, and a DA may let one class's signature substitute for another's. The Master versions need to feel clearly larger than the lower-tier versions.</t>
+          <t>A numeric DP column becomes mixed text/number, which breaks sorting, filtering and any automated DP check. The review workbooks normalize it to 0, but the source remains inconsistent.</t>
         </is>
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>Differentiate by time and scope: Intellect reads the immediate scene; Warden knows the quarry over a hunt. Make the Master investigation (Test the Hypothesis) clearly bigger than the one-minute version. State the intended overlap in the class guidance if it is deliberate.</t>
+          <t>Use DP 0 or leave DP blank and add an explicit 'Available to all' flag. Keep the numeric column numeric.</t>
         </is>
       </c>
       <c r="H33" s="10" t="inlineStr">
@@ -3006,42 +2980,42 @@
     <row r="34" ht="54" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>F32</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Universal</t>
+          <t>Ancestry</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>All 18 universal cards</t>
+          <t>Hard as Bedrock; Never Quite Finished; Grace of the Elder Folk; Adaptable</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>Universal cards store DP as the text 'Not purchased' instead of 0 or blank.</t>
+          <t>The baseline duplicate stat traits have been differentiated: Hard as Bedrock (+1 maximum HP), Never Quite Finished (+1 maximum HP and a death-mark Boon), Grace of the Elder Folk (+1 Speed) and Adaptable (+1 DP per level).</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>A numeric DP column becomes mixed text/number, which breaks sorting, filtering and any automated DP check. The review workbooks normalize it to 0, but the source remains inconsistent.</t>
+          <t>Ancestry stat choices now have distinct mechanical identities rather than two identical +1 HP/+1 Speed picks.</t>
         </is>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Use DP 0 or leave DP blank and add an explicit 'Available to all' flag. Keep the numeric column numeric.</t>
+          <t>No further action; keep the differentiation.</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr"/>
@@ -3149,15 +3123,12 @@
       <formula>J5="Cut"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3">
-      <formula>J5="Playtest"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="4">
       <formula>J5="Unsure"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J5:J36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Decision" error="Choose Keep, Revise, Cut, Playtest or Unsure." promptTitle="Decision" prompt="Your review decision for this row." type="list">
-      <formula1>"Keep,Revise,Cut,Playtest,Unsure"</formula1>
+    <dataValidation sqref="J5:J36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Decision" error="Choose Keep, Revise, Cut or Unsure." promptTitle="Decision" prompt="Your review decision for this row." type="list">
+      <formula1>"Keep,Revise,Cut,Unsure"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -3181,7 +3152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:K99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -6755,12 +6726,12 @@
     <row r="76" ht="29" customHeight="1">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>Arcane Deflection</t>
+          <t>Careful Transfer</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>signature-arcanist-arcane-deflection</t>
+          <t>signature-shepherd-careful-transfer</t>
         </is>
       </c>
       <c r="C76" s="11" t="inlineStr">
@@ -6770,7 +6741,7 @@
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Arcanist</t>
+          <t>Shepherd</t>
         </is>
       </c>
       <c r="E76" s="14" t="inlineStr">
@@ -6780,22 +6751,22 @@
       </c>
       <c r="F76" s="11" t="inlineStr">
         <is>
-          <t>2 Boons</t>
+          <t>Footnote placement</t>
         </is>
       </c>
       <c r="G76" s="11" t="inlineStr">
         <is>
-          <t>Reaction grants 2 Boons to a spell defense, above the usual 1.</t>
+          <t>Offensive healing exception is outside Rules.</t>
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr">
         <is>
-          <t>Confirm 2 is intended; compare to shared defense cards.</t>
+          <t>Move it into Rules or tag it.</t>
         </is>
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>signature-arcanist-arcane-deflection.md</t>
+          <t>signature-shepherd-careful-transfer.md</t>
         </is>
       </c>
       <c r="J76" s="11" t="inlineStr"/>
@@ -6804,12 +6775,12 @@
     <row r="77" ht="29" customHeight="1">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>Careful Transfer</t>
+          <t>Haul Them Home</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>signature-shepherd-careful-transfer</t>
+          <t>haul-them-home</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -6819,7 +6790,7 @@
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>Shepherd</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="E77" s="14" t="inlineStr">
@@ -6834,7 +6805,7 @@
       </c>
       <c r="G77" s="10" t="inlineStr">
         <is>
-          <t>Offensive healing exception is outside Rules.</t>
+          <t>Stability exception is outside Rules.</t>
         </is>
       </c>
       <c r="H77" s="10" t="inlineStr">
@@ -6844,7 +6815,7 @@
       </c>
       <c r="I77" s="10" t="inlineStr">
         <is>
-          <t>signature-shepherd-careful-transfer.md</t>
+          <t>haul-them-home.md</t>
         </is>
       </c>
       <c r="J77" s="10" t="inlineStr"/>
@@ -6853,12 +6824,12 @@
     <row r="78" ht="29" customHeight="1">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>Haul Them Home</t>
+          <t>Open the Way</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>haul-them-home</t>
+          <t>signature-shadow-open-the-way</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr">
@@ -6868,7 +6839,7 @@
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Shadow</t>
         </is>
       </c>
       <c r="E78" s="14" t="inlineStr">
@@ -6878,22 +6849,22 @@
       </c>
       <c r="F78" s="11" t="inlineStr">
         <is>
-          <t>Footnote placement</t>
+          <t>Niche signature</t>
         </is>
       </c>
       <c r="G78" s="11" t="inlineStr">
         <is>
-          <t>Stability exception is outside Rules.</t>
+          <t>Lockpicking at Adept; campaign-dependent.</t>
         </is>
       </c>
       <c r="H78" s="11" t="inlineStr">
         <is>
-          <t>Move it into Rules or tag it.</t>
+          <t>Add a trap/door clause or move to shared Subterfuge.</t>
         </is>
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>haul-them-home.md</t>
+          <t>signature-shadow-open-the-way.md</t>
         </is>
       </c>
       <c r="J78" s="11" t="inlineStr"/>
@@ -6902,12 +6873,12 @@
     <row r="79" ht="29" customHeight="1">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>Open the Way</t>
+          <t>Summon Animal — Adept</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>signature-shadow-open-the-way</t>
+          <t>call-the-hunting-cat</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
@@ -6917,7 +6888,7 @@
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>Shadow</t>
+          <t>Summon matrix</t>
         </is>
       </c>
       <c r="E79" s="14" t="inlineStr">
@@ -6927,22 +6898,22 @@
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t>Niche signature</t>
+          <t>Template family</t>
         </is>
       </c>
       <c r="G79" s="10" t="inlineStr">
         <is>
-          <t>Lockpicking at Adept; campaign-dependent.</t>
+          <t>One of 18 near-identical summon cards; title/ID/filename may not match.</t>
         </is>
       </c>
       <c r="H79" s="10" t="inlineStr">
         <is>
-          <t>Add a trap/door clause or move to shared Subterfuge.</t>
+          <t>Consolidate to a shared procedure plus six type records; align names.</t>
         </is>
       </c>
       <c r="I79" s="10" t="inlineStr">
         <is>
-          <t>signature-shadow-open-the-way.md</t>
+          <t>call-the-hunting-cat.md</t>
         </is>
       </c>
       <c r="J79" s="10" t="inlineStr"/>
@@ -6951,12 +6922,12 @@
     <row r="80" ht="29" customHeight="1">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>Summon Animal — Adept</t>
+          <t>Summon Construct — Adept</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>call-the-hunting-cat</t>
+          <t>the-walking-toolbox</t>
         </is>
       </c>
       <c r="C80" s="11" t="inlineStr">
@@ -6991,7 +6962,7 @@
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>call-the-hunting-cat.md</t>
+          <t>the-walking-toolbox.md</t>
         </is>
       </c>
       <c r="J80" s="11" t="inlineStr"/>
@@ -7000,12 +6971,12 @@
     <row r="81" ht="29" customHeight="1">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>Summon Construct — Adept</t>
+          <t>Summon Elemental — Adept</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>the-walking-toolbox</t>
+          <t>summon-elemental-adept</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -7040,7 +7011,7 @@
       </c>
       <c r="I81" s="10" t="inlineStr">
         <is>
-          <t>the-walking-toolbox.md</t>
+          <t>summon-elemental-adept.md</t>
         </is>
       </c>
       <c r="J81" s="10" t="inlineStr"/>
@@ -7049,12 +7020,12 @@
     <row r="82" ht="29" customHeight="1">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>Summon Elemental — Adept</t>
+          <t>Summon Fey — Adept</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>summon-elemental-adept</t>
+          <t>summon-fey-adept</t>
         </is>
       </c>
       <c r="C82" s="11" t="inlineStr">
@@ -7089,7 +7060,7 @@
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>summon-elemental-adept.md</t>
+          <t>summon-fey-adept.md</t>
         </is>
       </c>
       <c r="J82" s="11" t="inlineStr"/>
@@ -7098,12 +7069,12 @@
     <row r="83" ht="29" customHeight="1">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>Summon Fey — Adept</t>
+          <t>Summon Spirit — Adept</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>summon-fey-adept</t>
+          <t>call-a-sentinel</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
@@ -7138,7 +7109,7 @@
       </c>
       <c r="I83" s="10" t="inlineStr">
         <is>
-          <t>summon-fey-adept.md</t>
+          <t>call-a-sentinel.md</t>
         </is>
       </c>
       <c r="J83" s="10" t="inlineStr"/>
@@ -7147,12 +7118,12 @@
     <row r="84" ht="29" customHeight="1">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>Summon Spirit — Adept</t>
+          <t>Summon Undead — Adept</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>call-a-sentinel</t>
+          <t>summon-undead-adept</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
@@ -7187,7 +7158,7 @@
       </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>call-a-sentinel.md</t>
+          <t>summon-undead-adept.md</t>
         </is>
       </c>
       <c r="J84" s="11" t="inlineStr"/>
@@ -7196,12 +7167,12 @@
     <row r="85" ht="29" customHeight="1">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>Summon Undead — Adept</t>
+          <t>Sustain the Failing</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>summon-undead-adept</t>
+          <t>sustain-the-failing</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -7211,7 +7182,7 @@
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>Summon matrix</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="E85" s="14" t="inlineStr">
@@ -7221,22 +7192,22 @@
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t>Template family</t>
+          <t>Footnote placement</t>
         </is>
       </c>
       <c r="G85" s="10" t="inlineStr">
         <is>
-          <t>One of 18 near-identical summon cards; title/ID/filename may not match.</t>
+          <t>Offensive healing exception is outside Rules.</t>
         </is>
       </c>
       <c r="H85" s="10" t="inlineStr">
         <is>
-          <t>Consolidate to a shared procedure plus six type records; align names.</t>
+          <t>Move it into Rules or tag it.</t>
         </is>
       </c>
       <c r="I85" s="10" t="inlineStr">
         <is>
-          <t>summon-undead-adept.md</t>
+          <t>sustain-the-failing.md</t>
         </is>
       </c>
       <c r="J85" s="10" t="inlineStr"/>
@@ -7245,12 +7216,12 @@
     <row r="86" ht="29" customHeight="1">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>Sustain the Failing</t>
+          <t>Wind the Sight</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>sustain-the-failing</t>
+          <t>wind-the-sight</t>
         </is>
       </c>
       <c r="C86" s="11" t="inlineStr">
@@ -7270,22 +7241,22 @@
       </c>
       <c r="F86" s="11" t="inlineStr">
         <is>
-          <t>Footnote placement</t>
+          <t>Attack tag</t>
         </is>
       </c>
       <c r="G86" s="11" t="inlineStr">
         <is>
-          <t>Offensive healing exception is outside Rules.</t>
+          <t>Type Skill / Attack but makes no attack roll.</t>
         </is>
       </c>
       <c r="H86" s="11" t="inlineStr">
         <is>
-          <t>Move it into Rules or tag it.</t>
+          <t>Add a Setup tag.</t>
         </is>
       </c>
       <c r="I86" s="11" t="inlineStr">
         <is>
-          <t>sustain-the-failing.md</t>
+          <t>wind-the-sight.md</t>
         </is>
       </c>
       <c r="J86" s="11" t="inlineStr"/>
@@ -7294,22 +7265,22 @@
     <row r="87" ht="29" customHeight="1">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>Wind the Sight</t>
+          <t>Choose the Edge</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>wind-the-sight</t>
+          <t>signature-arcanist-choose-the-edge</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>Adept (level 3)</t>
+          <t>Master (level 7)</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Arcanist</t>
         </is>
       </c>
       <c r="E87" s="14" t="inlineStr">
@@ -7319,22 +7290,22 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t>Attack tag</t>
+          <t>Master feel</t>
         </is>
       </c>
       <c r="G87" s="10" t="inlineStr">
         <is>
-          <t>Type Skill / Attack but makes no attack roll.</t>
+          <t>2-square push on up to two targets; modest for a Master slot.</t>
         </is>
       </c>
       <c r="H87" s="10" t="inlineStr">
         <is>
-          <t>Add a Setup tag.</t>
+          <t>Consider a stronger rider or accept as a simple Master option.</t>
         </is>
       </c>
       <c r="I87" s="10" t="inlineStr">
         <is>
-          <t>wind-the-sight.md</t>
+          <t>signature-arcanist-choose-the-edge.md</t>
         </is>
       </c>
       <c r="J87" s="10" t="inlineStr"/>
@@ -7343,12 +7314,12 @@
     <row r="88" ht="29" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>Choose the Edge</t>
+          <t>Find the Seam</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>signature-arcanist-choose-the-edge</t>
+          <t>find-the-seam</t>
         </is>
       </c>
       <c r="C88" s="11" t="inlineStr">
@@ -7358,7 +7329,7 @@
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>Arcanist</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="E88" s="14" t="inlineStr">
@@ -7368,22 +7339,22 @@
       </c>
       <c r="F88" s="11" t="inlineStr">
         <is>
-          <t>Master feel</t>
+          <t>Attack tag</t>
         </is>
       </c>
       <c r="G88" s="11" t="inlineStr">
         <is>
-          <t>2-square push on up to two targets; modest for a Master slot.</t>
+          <t>Type Skill / Attack but makes no attack roll.</t>
         </is>
       </c>
       <c r="H88" s="11" t="inlineStr">
         <is>
-          <t>Consider a stronger rider or accept as a simple Master option.</t>
+          <t>Add a Setup tag.</t>
         </is>
       </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
-          <t>signature-arcanist-choose-the-edge.md</t>
+          <t>find-the-seam.md</t>
         </is>
       </c>
       <c r="J88" s="11" t="inlineStr"/>
@@ -7392,12 +7363,12 @@
     <row r="89" ht="29" customHeight="1">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>Find the Seam</t>
+          <t>Leave No Pursuit</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>find-the-seam</t>
+          <t>signature-shadow-leave-no-pursuit</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
@@ -7407,7 +7378,7 @@
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Shadow</t>
         </is>
       </c>
       <c r="E89" s="14" t="inlineStr">
@@ -7417,22 +7388,22 @@
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t>Attack tag</t>
+          <t>Niche signature</t>
         </is>
       </c>
       <c r="G89" s="10" t="inlineStr">
         <is>
-          <t>Type Skill / Attack but makes no attack roll.</t>
+          <t>Trail concealment at Master; campaign-dependent.</t>
         </is>
       </c>
       <c r="H89" s="10" t="inlineStr">
         <is>
-          <t>Add a Setup tag.</t>
+          <t>Accept as a specialist pick or add an ambush benefit.</t>
         </is>
       </c>
       <c r="I89" s="10" t="inlineStr">
         <is>
-          <t>find-the-seam.md</t>
+          <t>signature-shadow-leave-no-pursuit.md</t>
         </is>
       </c>
       <c r="J89" s="10" t="inlineStr"/>
@@ -7441,12 +7412,12 @@
     <row r="90" ht="29" customHeight="1">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>Leave No Pursuit</t>
+          <t>Perfect Placement</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>signature-shadow-leave-no-pursuit</t>
+          <t>signature-blade-perfect-placement</t>
         </is>
       </c>
       <c r="C90" s="11" t="inlineStr">
@@ -7456,7 +7427,7 @@
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Shadow</t>
+          <t>Blade</t>
         </is>
       </c>
       <c r="E90" s="14" t="inlineStr">
@@ -7466,22 +7437,22 @@
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>Niche signature</t>
+          <t>Master feel</t>
         </is>
       </c>
       <c r="G90" s="11" t="inlineStr">
         <is>
-          <t>Trail concealment at Master; campaign-dependent.</t>
+          <t>Push 2 then move 2; simple and similar to lower-tier movement riders.</t>
         </is>
       </c>
       <c r="H90" s="11" t="inlineStr">
         <is>
-          <t>Accept as a specialist pick or add an ambush benefit.</t>
+          <t>Consider push 3 or an ally movement clause.</t>
         </is>
       </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
-          <t>signature-shadow-leave-no-pursuit.md</t>
+          <t>signature-blade-perfect-placement.md</t>
         </is>
       </c>
       <c r="J90" s="11" t="inlineStr"/>
@@ -7490,12 +7461,12 @@
     <row r="91" ht="29" customHeight="1">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>Perfect Placement</t>
+          <t>Restore Composure</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>signature-blade-perfect-placement</t>
+          <t>signature-shepherd-restore-composure</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
@@ -7505,7 +7476,7 @@
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Blade</t>
+          <t>Shepherd</t>
         </is>
       </c>
       <c r="E91" s="14" t="inlineStr">
@@ -7515,22 +7486,22 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t>Master feel</t>
+          <t>Footnote placement</t>
         </is>
       </c>
       <c r="G91" s="10" t="inlineStr">
         <is>
-          <t>Push 2 then move 2; simple and similar to lower-tier movement riders.</t>
+          <t>Offensive healing exception is outside Rules.</t>
         </is>
       </c>
       <c r="H91" s="10" t="inlineStr">
         <is>
-          <t>Consider push 3 or an ally movement clause.</t>
+          <t>Move it into Rules or tag it.</t>
         </is>
       </c>
       <c r="I91" s="10" t="inlineStr">
         <is>
-          <t>signature-blade-perfect-placement.md</t>
+          <t>signature-shepherd-restore-composure.md</t>
         </is>
       </c>
       <c r="J91" s="10" t="inlineStr"/>
@@ -7539,12 +7510,12 @@
     <row r="92" ht="29" customHeight="1">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>Restore Composure</t>
+          <t>Return to Strength</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>signature-shepherd-restore-composure</t>
+          <t>return-to-strength</t>
         </is>
       </c>
       <c r="C92" s="11" t="inlineStr">
@@ -7554,7 +7525,7 @@
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>Shepherd</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="E92" s="14" t="inlineStr">
@@ -7579,7 +7550,7 @@
       </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
-          <t>signature-shepherd-restore-composure.md</t>
+          <t>return-to-strength.md</t>
         </is>
       </c>
       <c r="J92" s="11" t="inlineStr"/>
@@ -7588,12 +7559,12 @@
     <row r="93" ht="29" customHeight="1">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>Return to Strength</t>
+          <t>Strange but Effective</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>return-to-strength</t>
+          <t>signature-odd-strange-but-effective</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
@@ -7603,7 +7574,7 @@
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Odd</t>
         </is>
       </c>
       <c r="E93" s="14" t="inlineStr">
@@ -7613,22 +7584,22 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>Footnote placement</t>
+          <t>Missing numeral</t>
         </is>
       </c>
       <c r="G93" s="10" t="inlineStr">
         <is>
-          <t>Offensive healing exception is outside Rules.</t>
+          <t>Outcome lines say 'or squares of push' without a number.</t>
         </is>
       </c>
       <c r="H93" s="10" t="inlineStr">
         <is>
-          <t>Move it into Rules or tag it.</t>
+          <t>Write 2/3/4 squares of push.</t>
         </is>
       </c>
       <c r="I93" s="10" t="inlineStr">
         <is>
-          <t>return-to-strength.md</t>
+          <t>signature-odd-strange-but-effective.md</t>
         </is>
       </c>
       <c r="J93" s="10" t="inlineStr"/>
@@ -7637,12 +7608,12 @@
     <row r="94" ht="29" customHeight="1">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>Strange but Effective</t>
+          <t>Summon Animal — Master</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>signature-odd-strange-but-effective</t>
+          <t>call-the-elder-stag</t>
         </is>
       </c>
       <c r="C94" s="11" t="inlineStr">
@@ -7652,7 +7623,7 @@
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Odd</t>
+          <t>Summon matrix</t>
         </is>
       </c>
       <c r="E94" s="14" t="inlineStr">
@@ -7662,22 +7633,22 @@
       </c>
       <c r="F94" s="11" t="inlineStr">
         <is>
-          <t>Missing numeral</t>
+          <t>Template family</t>
         </is>
       </c>
       <c r="G94" s="11" t="inlineStr">
         <is>
-          <t>Outcome lines say 'or squares of push' without a number.</t>
+          <t>One of 18 near-identical summon cards; title/ID/filename may not match.</t>
         </is>
       </c>
       <c r="H94" s="11" t="inlineStr">
         <is>
-          <t>Write 2/3/4 squares of push.</t>
+          <t>Consolidate to a shared procedure plus six type records; align names.</t>
         </is>
       </c>
       <c r="I94" s="11" t="inlineStr">
         <is>
-          <t>signature-odd-strange-but-effective.md</t>
+          <t>call-the-elder-stag.md</t>
         </is>
       </c>
       <c r="J94" s="11" t="inlineStr"/>
@@ -7686,12 +7657,12 @@
     <row r="95" ht="29" customHeight="1">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>Summon Animal — Master</t>
+          <t>Summon Construct — Master</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>call-the-elder-stag</t>
+          <t>summon-construct-master</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
@@ -7726,7 +7697,7 @@
       </c>
       <c r="I95" s="10" t="inlineStr">
         <is>
-          <t>call-the-elder-stag.md</t>
+          <t>summon-construct-master.md</t>
         </is>
       </c>
       <c r="J95" s="10" t="inlineStr"/>
@@ -7735,12 +7706,12 @@
     <row r="96" ht="29" customHeight="1">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>Summon Construct — Master</t>
+          <t>Summon Elemental — Master</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>summon-construct-master</t>
+          <t>call-a-tempest-beast</t>
         </is>
       </c>
       <c r="C96" s="11" t="inlineStr">
@@ -7775,7 +7746,7 @@
       </c>
       <c r="I96" s="11" t="inlineStr">
         <is>
-          <t>summon-construct-master.md</t>
+          <t>call-a-tempest-beast.md</t>
         </is>
       </c>
       <c r="J96" s="11" t="inlineStr"/>
@@ -7784,12 +7755,12 @@
     <row r="97" ht="29" customHeight="1">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>Summon Elemental — Master</t>
+          <t>Summon Fey — Master</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>call-a-tempest-beast</t>
+          <t>summon-fey-master</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
@@ -7824,7 +7795,7 @@
       </c>
       <c r="I97" s="10" t="inlineStr">
         <is>
-          <t>call-a-tempest-beast.md</t>
+          <t>summon-fey-master.md</t>
         </is>
       </c>
       <c r="J97" s="10" t="inlineStr"/>
@@ -7833,12 +7804,12 @@
     <row r="98" ht="29" customHeight="1">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>Summon Fey — Master</t>
+          <t>Summon Spirit — Master</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>summon-fey-master</t>
+          <t>the-ancestors-stand</t>
         </is>
       </c>
       <c r="C98" s="11" t="inlineStr">
@@ -7873,7 +7844,7 @@
       </c>
       <c r="I98" s="11" t="inlineStr">
         <is>
-          <t>summon-fey-master.md</t>
+          <t>the-ancestors-stand.md</t>
         </is>
       </c>
       <c r="J98" s="11" t="inlineStr"/>
@@ -7882,12 +7853,12 @@
     <row r="99" ht="29" customHeight="1">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>Summon Spirit — Master</t>
+          <t>Summon Undead — Master</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>the-ancestors-stand</t>
+          <t>procession-of-the-quiet</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -7922,68 +7893,19 @@
       </c>
       <c r="I99" s="10" t="inlineStr">
         <is>
-          <t>the-ancestors-stand.md</t>
+          <t>procession-of-the-quiet.md</t>
         </is>
       </c>
       <c r="J99" s="10" t="inlineStr"/>
       <c r="K99" s="10" t="inlineStr"/>
     </row>
-    <row r="100" ht="29" customHeight="1">
-      <c r="A100" s="11" t="inlineStr">
-        <is>
-          <t>Summon Undead — Master</t>
-        </is>
-      </c>
-      <c r="B100" s="11" t="inlineStr">
-        <is>
-          <t>procession-of-the-quiet</t>
-        </is>
-      </c>
-      <c r="C100" s="11" t="inlineStr">
-        <is>
-          <t>Master (level 7)</t>
-        </is>
-      </c>
-      <c r="D100" s="11" t="inlineStr">
-        <is>
-          <t>Summon matrix</t>
-        </is>
-      </c>
-      <c r="E100" s="14" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F100" s="11" t="inlineStr">
-        <is>
-          <t>Template family</t>
-        </is>
-      </c>
-      <c r="G100" s="11" t="inlineStr">
-        <is>
-          <t>One of 18 near-identical summon cards; title/ID/filename may not match.</t>
-        </is>
-      </c>
-      <c r="H100" s="11" t="inlineStr">
-        <is>
-          <t>Consolidate to a shared procedure plus six type records; align names.</t>
-        </is>
-      </c>
-      <c r="I100" s="11" t="inlineStr">
-        <is>
-          <t>procession-of-the-quiet.md</t>
-        </is>
-      </c>
-      <c r="J100" s="11" t="inlineStr"/>
-      <c r="K100" s="11" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:J100"/>
+  <autoFilter ref="A4:J99"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="J5:J100">
+  <conditionalFormatting sqref="J5:J99">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>J5="Keep"</formula>
     </cfRule>
@@ -7994,15 +7916,12 @@
       <formula>J5="Cut"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3">
-      <formula>J5="Playtest"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="4">
       <formula>J5="Unsure"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J5:J100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Decision" error="Choose Keep, Revise, Cut, Playtest or Unsure." promptTitle="Decision" prompt="Your review decision for this row." type="list">
-      <formula1>"Keep,Revise,Cut,Playtest,Unsure"</formula1>
+    <dataValidation sqref="J5:J99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Decision" error="Choose Keep, Revise, Cut or Unsure." promptTitle="Decision" prompt="Your review decision for this row." type="list">
+      <formula1>"Keep,Revise,Cut,Unsure"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -8026,7 +7945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8041,12 +7960,11 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" style="16" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" style="16" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -8127,30 +8045,25 @@
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>Playtest status</t>
+          <t>Book issue</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
         <is>
-          <t>Book issue</t>
+          <t>Foundry issue</t>
         </is>
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t>Foundry issue</t>
+          <t>Commit SHA</t>
         </is>
       </c>
       <c r="P4" s="6" t="inlineStr">
         <is>
-          <t>Commit SHA</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="Q4" s="6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="R4" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -8174,7 +8087,6 @@
       <c r="O5" s="10" t="inlineStr"/>
       <c r="P5" s="10" t="inlineStr"/>
       <c r="Q5" s="10" t="inlineStr"/>
-      <c r="R5" s="10" t="inlineStr"/>
     </row>
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="11" t="inlineStr"/>
@@ -8194,7 +8106,6 @@
       <c r="O6" s="11" t="inlineStr"/>
       <c r="P6" s="11" t="inlineStr"/>
       <c r="Q6" s="11" t="inlineStr"/>
-      <c r="R6" s="11" t="inlineStr"/>
     </row>
     <row r="7" ht="16.5" customHeight="1">
       <c r="A7" s="10" t="inlineStr"/>
@@ -8214,7 +8125,6 @@
       <c r="O7" s="10" t="inlineStr"/>
       <c r="P7" s="10" t="inlineStr"/>
       <c r="Q7" s="10" t="inlineStr"/>
-      <c r="R7" s="10" t="inlineStr"/>
     </row>
     <row r="8" ht="16.5" customHeight="1">
       <c r="A8" s="11" t="inlineStr"/>
@@ -8234,7 +8144,6 @@
       <c r="O8" s="11" t="inlineStr"/>
       <c r="P8" s="11" t="inlineStr"/>
       <c r="Q8" s="11" t="inlineStr"/>
-      <c r="R8" s="11" t="inlineStr"/>
     </row>
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="10" t="inlineStr"/>
@@ -8254,7 +8163,6 @@
       <c r="O9" s="10" t="inlineStr"/>
       <c r="P9" s="10" t="inlineStr"/>
       <c r="Q9" s="10" t="inlineStr"/>
-      <c r="R9" s="10" t="inlineStr"/>
     </row>
     <row r="10" ht="16.5" customHeight="1">
       <c r="A10" s="11" t="inlineStr"/>
@@ -8274,7 +8182,6 @@
       <c r="O10" s="11" t="inlineStr"/>
       <c r="P10" s="11" t="inlineStr"/>
       <c r="Q10" s="11" t="inlineStr"/>
-      <c r="R10" s="11" t="inlineStr"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="10" t="inlineStr"/>
@@ -8294,7 +8201,6 @@
       <c r="O11" s="10" t="inlineStr"/>
       <c r="P11" s="10" t="inlineStr"/>
       <c r="Q11" s="10" t="inlineStr"/>
-      <c r="R11" s="10" t="inlineStr"/>
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="11" t="inlineStr"/>
@@ -8314,7 +8220,6 @@
       <c r="O12" s="11" t="inlineStr"/>
       <c r="P12" s="11" t="inlineStr"/>
       <c r="Q12" s="11" t="inlineStr"/>
-      <c r="R12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="10" t="inlineStr"/>
@@ -8334,7 +8239,6 @@
       <c r="O13" s="10" t="inlineStr"/>
       <c r="P13" s="10" t="inlineStr"/>
       <c r="Q13" s="10" t="inlineStr"/>
-      <c r="R13" s="10" t="inlineStr"/>
     </row>
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="11" t="inlineStr"/>
@@ -8354,7 +8258,6 @@
       <c r="O14" s="11" t="inlineStr"/>
       <c r="P14" s="11" t="inlineStr"/>
       <c r="Q14" s="11" t="inlineStr"/>
-      <c r="R14" s="11" t="inlineStr"/>
     </row>
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="10" t="inlineStr"/>
@@ -8374,7 +8277,6 @@
       <c r="O15" s="10" t="inlineStr"/>
       <c r="P15" s="10" t="inlineStr"/>
       <c r="Q15" s="10" t="inlineStr"/>
-      <c r="R15" s="10" t="inlineStr"/>
     </row>
     <row r="16" ht="16.5" customHeight="1">
       <c r="A16" s="11" t="inlineStr"/>
@@ -8394,23 +8296,19 @@
       <c r="O16" s="11" t="inlineStr"/>
       <c r="P16" s="11" t="inlineStr"/>
       <c r="Q16" s="11" t="inlineStr"/>
-      <c r="R16" s="11" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:R204"/>
+  <autoFilter ref="A4:Q204"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation sqref="I5:I204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Change type" error="Choose one of: Editorial, Wording, Mechanical, Rename, Add, Remove, Tier / DP, ID migration" promptTitle="Change type" prompt="Classify the change." type="list">
       <formula1>"Editorial,Wording,Mechanical,Rename,Add,Remove,Tier / DP,ID migration"</formula1>
     </dataValidation>
     <dataValidation sqref="K5:K204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Decision" error="Choose one of: Proposed, Approved, Rejected, Deferred" promptTitle="Decision" prompt="Approval state for this change." type="list">
       <formula1>"Proposed,Approved,Rejected,Deferred"</formula1>
-    </dataValidation>
-    <dataValidation sqref="M5:M204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Playtest status" error="Choose one of: Not needed, Pending, Passed, Failed, N/A" promptTitle="Playtest status" prompt="Playtest evidence for mechanical changes." type="list">
-      <formula1>"Not needed,Pending,Passed,Failed,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -9043,7 +8941,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="54" customHeight="1">
+    <row r="26" ht="91.5" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Dwarf</t>
@@ -9069,16 +8967,16 @@
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>Stubborn as Bedrock</t>
+          <t>Hard as Bedrock</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>Stubborn as Bedrock is a bare +1 HP. Maker's Hand and Mountain Remembers are narrow and partly overlap. The ancestry has no social or movement trait, so it can feel one-note outside combat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="54" customHeight="1">
+          <t>Hard as Bedrock is intentionally a bare +1 HP; it is the simple durability pick, not a trait with a dramatic moment. Maker's Hand covers portable items and workmanship; Stone Mason covers structures, stone crafting and structural weakness. The ancestry has no social or movement trait, so it can feel one-note outside combat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="66.5" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Elf</t>
@@ -9109,11 +9007,11 @@
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>Several traits are woodland- or rest-specific; A Lifetime Ago needs campaign buy-in. Grace is mechanically identical to Human Road in the Blood. The ancestry has no social trait beyond lore.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="54" customHeight="1">
+          <t>Footfall is strong in woodland but does nothing outside it; several other traits are woodland- or rest-specific. A Lifetime Ago is broad but limited to once per day. Grace is the straightforward +1 Speed option. The ancestry has no social trait beyond lore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="41.5" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Halfling</t>
@@ -9144,11 +9042,11 @@
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>No trait raises HP or Speed, and base HP/Speed are the lowest. Second Breakfast is mechanically thin. Bigger on the Inside is niche unless fear is common. Halfling is the only ancestry with no stat trait.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="54" customHeight="1">
+          <t>Base HP/Speed are the lowest. Bigger on the Inside now covers HP, but the ancestry still has no Speed trait. Endless Pockets is a small utility benefit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="41.5" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Human</t>
@@ -9174,12 +9072,12 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Never Quite Finished, Road in the Blood</t>
+          <t>Never Quite Finished</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>Never Quite Finished and Road in the Blood duplicate Dwarf/Elf stat traits. The travel clause on Road is mostly flavor because there is no exhaustion rule. The Impossible Streak may overshadow skill-focused classes.</t>
+          <t>Adaptable is a strong character-building advantage rather than a scene ability. The Impossible Streak may overshadow skill-focused classes.</t>
         </is>
       </c>
     </row>

</xml_diff>